<commit_message>
Updated to Version 3.0.0
</commit_message>
<xml_diff>
--- a/Test_BI_Analysis_Report_2026.xlsx
+++ b/Test_BI_Analysis_Report_2026.xlsx
@@ -1548,22 +1548,55 @@
       <c r="B20" s="3" t="n">
         <v>46281</v>
       </c>
-      <c r="C20" s="2" t="n"/>
-      <c r="D20" s="2" t="n"/>
-      <c r="E20" s="2" t="n"/>
-      <c r="F20" s="2" t="n"/>
-      <c r="G20" s="2" t="n"/>
-      <c r="H20" s="2" t="n"/>
-      <c r="I20" s="2" t="n"/>
-      <c r="J20" s="2" t="n"/>
-      <c r="K20" s="2" t="n"/>
-      <c r="L20" s="2" t="n"/>
-      <c r="M20" s="2" t="n"/>
-      <c r="N20" s="2" t="n"/>
-      <c r="O20" s="2" t="n"/>
-      <c r="P20" s="2" t="n"/>
-      <c r="Q20" s="2" t="n"/>
-      <c r="R20" s="2" t="n"/>
+      <c r="C20" s="13" t="n">
+        <v>3420.54</v>
+      </c>
+      <c r="D20" s="13" t="n">
+        <v>66.09999999999999</v>
+      </c>
+      <c r="E20" s="13" t="n">
+        <v>504.68</v>
+      </c>
+      <c r="F20" s="13" t="n">
+        <v>171.81</v>
+      </c>
+      <c r="G20" s="13" t="n">
+        <v>1039.61</v>
+      </c>
+      <c r="H20" s="13" t="n">
+        <v>1975.17</v>
+      </c>
+      <c r="I20" s="13" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="J20" s="13" t="n">
+        <v>193.03</v>
+      </c>
+      <c r="K20" s="13" t="n">
+        <v>773.41</v>
+      </c>
+      <c r="L20" s="13" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="M20" s="13" t="n">
+        <v>1023.72</v>
+      </c>
+      <c r="N20" s="13" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="O20" s="13" t="n">
+        <v>263.22</v>
+      </c>
+      <c r="P20" s="13" t="n">
+        <v>17.66</v>
+      </c>
+      <c r="Q20" s="13" t="n">
+        <v>149.81</v>
+      </c>
+      <c r="R20" s="13">
+        <f>SUM(C20:Q20)</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="B21" s="3" t="n">

</xml_diff>